<commit_message>
Add UP_02 v2.0 iteration and update parts
</commit_message>
<xml_diff>
--- a/FST16_DT_Parts_Export.xlsx
+++ b/FST16_DT_Parts_Export.xlsx
@@ -131,8 +131,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsTable" displayName="PartsTable" ref="A1:I37" headerRowCount="1">
-  <autoFilter ref="A1:I37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsTable" displayName="PartsTable" ref="A1:I38" headerRowCount="1">
+  <autoFilter ref="A1:I38"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Subassembly"/>
     <tableColumn id="2" name="Part Name"/>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1837,31 +1837,35 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>UP_03</t>
+          <t>UP_02</t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t>FST15</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>2026-10-06 11:18:14</t>
+          <t>2026-10-13 18:49:48</t>
         </is>
       </c>
       <c r="E36" s="1" t="n">
-        <v>59.37</v>
+        <v>122.76</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Flor FST15</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr"/>
+          <t>This version has all the features</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Transmission: v2.0</t>
+        </is>
+      </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>images\UP_03_vFST15_imagem.png</t>
+          <t>images/UP_02_v2_0_imagem.png</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -1874,30 +1878,67 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>UpperSupport Version</t>
+          <t>UP_03</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>FST15</t>
         </is>
       </c>
       <c r="D37" s="1" t="inlineStr">
         <is>
-          <t>2026-10-12 15:47:39</t>
+          <t>2026-10-06 11:18:14</t>
         </is>
       </c>
       <c r="E37" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="2" t="inlineStr"/>
+        <v>59.37</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Flor FST15</t>
+        </is>
+      </c>
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="inlineStr">
         <is>
+          <t>images\UP_03_vFST15_imagem.png</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>UpperSupport Version</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-12 15:47:39</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
           <t>images\UpperSupport Version_v1_0_imagem.png</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update fixed constraints for bearing 61816 from datasheet
</commit_message>
<xml_diff>
--- a/FST16_DT_Parts_Export.xlsx
+++ b/FST16_DT_Parts_Export.xlsx
@@ -1144,16 +1144,36 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Schaeffler Bearing: 61816
-Datasheet: 61816</t>
+          <t xml:space="preserve">Schaeffler Bearing: 61816  
+Datasheet: https://medias.schaeffler.es/pt/produto/rotary/rolamentos%2c-mancais-de-deslizamento/rolamentos-de-esferas/rolamentos-rigidos-de-esferas/61816/p/2893831#Product%20Information </t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Inner D (mm): 80 | Dynamic Load Cr (kN): 13.8 | Static Load C0r (kN): 13.8 | Speed Limit (rpm): 9400</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr"/>
+          <t>d (Diâmetro do furo): 80 mm
+D (Diâmetro externo): 100 mm
+B (Width / Largura): 10 mm
+Cr (Capacidade de carga dinâmica, radial): 13.800 N
+C0r (Capacidade de carga estática, radial): 13.800 N
+Cur (Limite de carga por fadiga, radial): 930 N
+nG (Velocidade limite): 9.400 1/min
+n_ref (Velocidade nominal): 4.600 1/min
+da min (Diâmetro mín. ressalto do veio): 83,2 mm
+Da max (Diâmetro máx. ressalto da casquilho): 96,8 mm
+ra max (Raio máximo da ranhura): 0,6 mm
+rmin (Minimum chamfer dimension): 0,6 mm
+D1 (Diâmetro do ressalto do anel exterior): 93,57 mm
+d1 (Diâmetro do ressalto do anel interior): 86,6 mm
+Tmin (Temperatura de operação min.): -30 °C
+Tmax (Temperatura de operação max.): 150 °C
+f0 (Fator de cálculo): 16</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>images/61816_vOEM_20261017_103218.png</t>
+        </is>
+      </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update drivetrain tracker data and web portal
</commit_message>
<xml_diff>
--- a/FST16_DT_Parts_Export.xlsx
+++ b/FST16_DT_Parts_Export.xlsx
@@ -131,8 +131,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsTable" displayName="PartsTable" ref="A1:L46" headerRowCount="1">
-  <autoFilter ref="A1:L46"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsTable" displayName="PartsTable" ref="A1:L47" headerRowCount="1">
+  <autoFilter ref="A1:L47"/>
   <tableColumns count="12">
     <tableColumn id="1" name="Subassembly"/>
     <tableColumn id="2" name="Part Name"/>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -808,30 +808,39 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>2026-10-07 13:36:53</t>
+          <t>2026-10-24 19:37:08</t>
         </is>
       </c>
       <c r="E8" s="1" t="n">
-        <v>596.3200000000001</v>
+        <v>618.5</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>the difference to 1.0 is due to missing the interface for the sleeve</t>
+          <t xml:space="preserve">The first iteration of the FST16 hub
+</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>images\HB_01_v1_1_imagem.png</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+          <t>images/HB_01_v5_0_20261024_193708.png</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>{"LC1": 0.03341, "LC2": 0.02446, "LC3": 0.22401, "LC4": 0.16215, "LC5": 0.13324, "LC6": 0.11568, "LC7": 0.15095}</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>{"LC1": "images/HB_01_v5_0_LC1_20261024_193900.png", "LC2": "images/HB_01_v5_0_LC2_20261024_193900.png", "LC3": "images/HB_01_v5_0_LC3_20261024_193900.png", "LC4": "images/HB_01_v5_0_LC4_20261024_193900.png", "LC5": "images/HB_01_v5_0_LC5_20261024_193900.png", "LC6": "images/HB_01_v5_0_LC6_20261024_193900.png", "LC7": "images/HB_01_v5_0_LC7_20261024_193900.png"}</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
     </row>
@@ -2678,35 +2687,49 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>UP_02</t>
+          <t>UP_01</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t>FST15</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="D41" s="1" t="inlineStr">
         <is>
-          <t>2026-10-06 11:18:14</t>
+          <t>2026-10-24 17:30:49</t>
         </is>
       </c>
       <c r="E41" s="1" t="n">
-        <v>114.52</v>
+        <v>1060.69</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Upright Lid FST15</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr"/>
+          <t xml:space="preserve">Corte no LowerSupport e aumento da largura do tierod
+</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Transmission: v5.0
+Bodies: 1</t>
+        </is>
+      </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>images\UP_02_vFST15_imagem.png</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="2" t="inlineStr"/>
+          <t>images/UP_01_v6_0_20261024_173049.png</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>{"LC1": 0.1536, "LC2": 0.179, "LC3": 0.2967, "LC4": 0.0, "LC5": 0.0, "LC6": 0.0, "LC7": 0.0, "LC8": 0.0648, "LC9": 0.0648}</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>{"LC1": "images/UP_01_v6_0_LC1_20261024_173049.png", "LC2": "images/UP_01_v6_0_LC2_20261024_173049.png", "LC3": "images/UP_01_v6_0_LC3_20261024_173049.png", "LC8": "images/UP_01_v6_0_LC8_20261024_173049.png", "LC9": "images/UP_01_v6_0_LC9_20261024_173049.png"}</t>
+        </is>
+      </c>
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr"/>
     </row>
@@ -2723,26 +2746,26 @@
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>FST15</t>
         </is>
       </c>
       <c r="D42" s="1" t="inlineStr">
         <is>
-          <t>2026-10-06 18:49:19</t>
+          <t>2026-10-06 11:18:14</t>
         </is>
       </c>
       <c r="E42" s="1" t="n">
-        <v>101.15</v>
+        <v>114.52</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Due to the less height is lighter</t>
+          <t>Upright Lid FST15</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>images\UP_02_v1_imagem.png</t>
+          <t>images\UP_02_vFST15_imagem.png</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2763,26 +2786,26 @@
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
-          <t>FST15 (with all features)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D43" s="1" t="inlineStr">
         <is>
-          <t>2026-10-13 20:39:47</t>
+          <t>2026-10-06 18:49:19</t>
         </is>
       </c>
       <c r="E43" s="1" t="n">
-        <v>120.04</v>
-      </c>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Transmission: v2.0</t>
-        </is>
-      </c>
+        <v>101.15</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Due to the less height is lighter</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>images/UP_02_vFST15 (with all features)_20261013_203947.png</t>
+          <t>images\UP_02_v1_imagem.png</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
@@ -2803,22 +2826,18 @@
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t>2.0 (with all features)</t>
+          <t>FST15 (with all features)</t>
         </is>
       </c>
       <c r="D44" s="1" t="inlineStr">
         <is>
-          <t>2026-10-13 20:48:17</t>
+          <t>2026-10-13 20:39:47</t>
         </is>
       </c>
       <c r="E44" s="1" t="n">
-        <v>116.27</v>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Corrected dimensions and features</t>
-        </is>
-      </c>
+        <v>120.04</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Transmission: v2.0</t>
@@ -2826,7 +2845,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>images/UP_02_v2_0 (with all features)_20261013_204817.png</t>
+          <t>images/UP_02_vFST15 (with all features)_20261013_203947.png</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2842,38 +2861,82 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>UP_03</t>
+          <t>UP_02</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>FST15</t>
+          <t>2.0 (with all features)</t>
         </is>
       </c>
       <c r="D45" s="1" t="inlineStr">
         <is>
-          <t>2026-10-06 11:18:14</t>
+          <t>2026-10-13 20:48:17</t>
         </is>
       </c>
       <c r="E45" s="1" t="n">
-        <v>59.37</v>
+        <v>116.27</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">To represent the FST15 part
-</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr"/>
+          <t>Corrected dimensions and features</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Transmission: v2.0</t>
+        </is>
+      </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>images\UP_03_vFST15_imagem.png</t>
+          <t>images/UP_02_v2_0 (with all features)_20261013_204817.png</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>UP_03</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>FST15</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-06 11:18:14</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>59.37</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">To represent the FST15 part
+</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>images\UP_03_vFST15_imagem.png</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>### Front Plate Trade Study
 #### 1. Summary &amp; Context
@@ -2966,50 +3029,50 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="1" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B46" s="1" t="inlineStr">
+      <c r="B47" s="1" t="inlineStr">
         <is>
           <t>UP_04</t>
         </is>
       </c>
-      <c r="C46" s="1" t="inlineStr">
+      <c r="C47" s="1" t="inlineStr">
         <is>
           <t>FST15</t>
         </is>
       </c>
-      <c r="D46" s="1" t="inlineStr">
+      <c r="D47" s="1" t="inlineStr">
         <is>
           <t>2026-10-17 11:42:38</t>
         </is>
       </c>
-      <c r="E46" s="1" t="n">
+      <c r="E47" s="1" t="n">
         <v>40.02</v>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Baseline motor back plate iteration for FST15 carry-over.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Radial O-Ring: 
 Axial O-Ring: </t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>images/UP_04_vFST15_20261017_114238.png</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr"/>
-      <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>### Backplate Rationale
 #### Component Trade-Off Study: Back Plate

</xml_diff>